<commit_message>
Update contact list with additional companies from directory search (72 contacts, 40 companies)
Added East Texas Roof Works, Evolution Roofing, BXC Roofing, Texas Roof Masters,
Accurate Roof Systems, CXR Roofing, Roof Care, Smith Roofing, Hail King, Sky High,
Calvary Roofing, Myers Roofing, plus additional employees at Tyler Roofing Company.

https://claude.ai/code/session_019vJRSZ4rBkhi5FH5Wtx4Bj
</commit_message>
<xml_diff>
--- a/output/Smith_County_TX_Roofing_Contacts.xlsx
+++ b/output/Smith_County_TX_Roofing_Contacts.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Roofing Contacts Smith Co TX" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roofing Contacts Smith Co TX'!$A$1:$G$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roofing Contacts Smith Co TX'!$A$1:$G$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1779,28 +1779,28 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Cris</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Weaver</t>
+          <t>Sukiennik</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>(903) 592-5892</t>
+          <t>(903) 597-4152</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Weaver Action Roofing Company</t>
+          <t>Tyler Roofing Company Inc.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Owner / President</t>
+          <t>General Manager</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -1812,28 +1812,28 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Janet</t>
+          <t>Tracy</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Weaver</t>
+          <t>Sukiennik</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>(903) 592-5892</t>
+          <t>(903) 597-4152</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Weaver Action Roofing Company</t>
+          <t>Tyler Roofing Company Inc.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Office Manager</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -1845,60 +1845,56 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Steve</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Rohus</t>
+          <t>Weaver</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>(903) 839-2060</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>steverohus@gmail.com</t>
-        </is>
-      </c>
+          <t>(903) 592-5892</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Steve's Quality Roofing</t>
+          <t>Weaver Action Roofing Company</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Owner / President</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Whitehouse</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Cori</t>
+          <t>Janet</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Moore</t>
+          <t>Weaver</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>(903) 534-3979</t>
+          <t>(903) 592-5892</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Project One Roofing</t>
+          <t>Weaver Action Roofing Company</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1908,63 +1904,63 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Whitehouse</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>John Oliver</t>
+          <t>Dewayne</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Boyd II</t>
+          <t>Gordon</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>(903) 810-7770</t>
+          <t>(903) 526-7419</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Boyd's of Texas</t>
+          <t>East Texas Roof Works &amp; Sheet Metal</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
+          <t>Owner / Founder</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Bullard</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Kurt</t>
+          <t>Steve</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Coleman</t>
+          <t>DeRaad</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>(903) 530-0350</t>
+          <t>(903) 526-7419</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr"/>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Coleman Roofing</t>
+          <t>East Texas Roof Works &amp; Sheet Metal</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -1981,23 +1977,23 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Dayton</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Longfellow</t>
+          <t>Gordon</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>(903) 245-2988</t>
+          <t>(903) 526-7419</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Goodfella's Roofing</t>
+          <t>East Texas Roof Works &amp; Sheet Metal</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2007,63 +2003,63 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Whitehouse</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Cody</t>
+          <t>Barbara</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Savell</t>
+          <t>Gordon</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>(903) 363-4140</t>
+          <t>(903) 526-7419</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr"/>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Bad Bear Roofing &amp; Construction</t>
+          <t>East Texas Roof Works &amp; Sheet Metal</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Corporate Secretary</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Roy</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Drewett</t>
+          <t>Rhodes</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>(903) 724-1511</t>
+          <t>(903) 258-1210</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Premier Roofing ETX</t>
+          <t>Evolution Roofing LLC</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2078,70 +2074,874 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr"/>
-      <c r="B47" s="2" t="inlineStr"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Zachary</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Reilly</t>
+        </is>
+      </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>(903) 969-0503</t>
+          <t>(903) 258-1210</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
+          <t>Evolution Roofing LLC</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Co-Owner</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Blake</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Wilabay</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>(903) 320-3030</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>bxcroofing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>BXC Roofing LLC</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Amelia</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Pratka</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>(903) 787-9043</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Info@roofmasterstyler.com</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Texas Roof Masters Tyler LLC</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Owner / Founder</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Spencer</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>(903) 894-6418</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Accurate Roof Systems</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Co-Owner / Founder</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Flint</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Melissa</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Spencer</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>(903) 894-6418</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Accurate Roof Systems</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Co-Owner</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Flint</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Jimenez</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>(903) 894-6418</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Accurate Roof Systems</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Director of Marketing</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Flint</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Zach</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Reilly</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>(903) 258-1210</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>office.cxrroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>CXR Roofing</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Ricardo</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Gamboa</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>(903) 399-5403</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>contact@roof.care</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Roof Care Inc.</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Michelle</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Gamboa</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>(903) 399-5403</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>contact@roof.care</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Roof Care Inc.</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Operations Director</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Chris</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Smith</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>(903) 279-7000</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Smith Roofing and Construction</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Landon</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Stokes</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>(682) 235-2880</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Hail King Professional Roofing LLC</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Co-Owner</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Lori</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Anderson-Stokes</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>(682) 235-2880</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Hail King Professional Roofing LLC</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Co-Owner</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Roman</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Skylar</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr"/>
+      <c r="D59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Sky High Roofing</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Hugo</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Escobar</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Sky High Roofing</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Nick</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr"/>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>(903) 714-3729</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Calvary Roofing and Construction</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Lindale</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr"/>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>(903) 714-3729</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Calvary Roofing and Construction</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Co-Owner</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Lindale</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Ronnie</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Myers</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>(903) 573-3431</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>RonMyersRoofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Myers Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Lindale</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Steve</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Rohus</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>(903) 839-2060</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>steverohus@gmail.com</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Steve's Quality Roofing</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Whitehouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Cori</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Moore</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>(903) 534-3979</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Project One Roofing</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Co-Owner</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Whitehouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>John Oliver</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Boyd II</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>(903) 810-7770</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Boyd's of Texas</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Bullard</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Kurt</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Coleman</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>(903) 530-0350</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr"/>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Coleman Roofing</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Dayton</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Longfellow</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>(903) 245-2988</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Goodfella's Roofing</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Whitehouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Cody</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Savell</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>(903) 363-4140</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr"/>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Bad Bear Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Flint</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Roy</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Drewett</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>(903) 724-1511</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Premier Roofing ETX</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr"/>
+      <c r="B71" s="2" t="inlineStr"/>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>(903) 969-0503</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr"/>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
           <t>ETX Roofing &amp; Construction</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr">
         <is>
           <t>Troup</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr"/>
-      <c r="B48" s="2" t="inlineStr"/>
-      <c r="C48" s="2" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr"/>
+      <c r="B72" s="2" t="inlineStr"/>
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>(903) 939-3168</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr"/>
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>Advantage Roofing</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>Tyler</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
-      <c r="B49" s="2" t="inlineStr"/>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr"/>
+      <c r="B73" s="2" t="inlineStr"/>
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>(903) 343-5700</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr"/>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr"/>
+      <c r="E73" s="2" t="inlineStr">
         <is>
           <t>ValueGuard Roofing</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr">
         <is>
           <t>Flint</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G49"/>
+  <autoFilter ref="A1:G73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Final update: add Cook & Son, Texas Direct, Roof Maxx, AVCO/Advantage names (78 contacts, 43 companies)
https://claude.ai/code/session_019vJRSZ4rBkhi5FH5Wtx4Bj
</commit_message>
<xml_diff>
--- a/output/Smith_County_TX_Roofing_Contacts.xlsx
+++ b/output/Smith_County_TX_Roofing_Contacts.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Roofing Contacts Smith Co TX" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roofing Contacts Smith Co TX'!$A$1:$G$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roofing Contacts Smith Co TX'!$A$1:$G$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1911,28 +1911,28 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Dewayne</t>
+          <t>A.J.</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Gordon</t>
+          <t>Cook III</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>(903) 526-7419</t>
+          <t>(903) 595-4567</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>East Texas Roof Works &amp; Sheet Metal</t>
+          <t>Cook and Son Roofing LLC</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Owner / Founder</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -1944,28 +1944,28 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Steve</t>
+          <t>Moriah</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>DeRaad</t>
+          <t>McClinton</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>(903) 526-7419</t>
+          <t>(903) 595-4567</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr"/>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>East Texas Roof Works &amp; Sheet Metal</t>
+          <t>Cook and Son Roofing LLC</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Secretary</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -1977,28 +1977,32 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Jimmy</t>
+          <t>Stephanie</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Gordon</t>
+          <t>Osborn</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>(903) 526-7419</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr"/>
+          <t>(903) 534-8700</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>office@avcoroofing.com</t>
+        </is>
+      </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>East Texas Roof Works &amp; Sheet Metal</t>
+          <t>AVCO Roofing</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Chief Operations Officer</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2010,28 +2014,28 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Barbara</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Gordon</t>
+          <t>Merrell</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>(903) 526-7419</t>
+          <t>(903) 939-3168</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr"/>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>East Texas Roof Works &amp; Sheet Metal</t>
+          <t>Advantage Roofing Company</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Corporate Secretary</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -2043,23 +2047,23 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Matthew Hunter</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Rhodes</t>
+          <t>Andrews</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>(903) 258-1210</t>
+          <t>(903) 710-4022</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Evolution Roofing LLC</t>
+          <t>Texas Direct Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2076,28 +2080,28 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Zachary</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Reilly</t>
+          <t>Stephens</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>(903) 258-1210</t>
+          <t>(903) 710-4022</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Evolution Roofing LLC</t>
+          <t>Texas Direct Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Director of Marketing</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -2109,32 +2113,32 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Blake</t>
+          <t>Greg</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Wilabay</t>
+          <t>Tryon</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>(903) 320-3030</t>
+          <t>(903) 752-7177</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>bxcroofing@yahoo.com</t>
+          <t>gtryon@roofmaxx.com</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>BXC Roofing LLC</t>
+          <t>Roof Maxx of Tyler</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2146,27 +2150,23 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Amelia</t>
+          <t>Dewayne</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Pratka</t>
+          <t>Gordon</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>(903) 787-9043</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Info@roofmasterstyler.com</t>
-        </is>
-      </c>
+          <t>(903) 526-7419</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr"/>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Texas Roof Masters Tyler LLC</t>
+          <t>East Texas Roof Works &amp; Sheet Metal</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2183,111 +2183,111 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Gabriel</t>
+          <t>Steve</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Spencer</t>
+          <t>DeRaad</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>(903) 894-6418</t>
+          <t>(903) 526-7419</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr"/>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Accurate Roof Systems</t>
+          <t>East Texas Roof Works &amp; Sheet Metal</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner / Founder</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Melissa</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Spencer</t>
+          <t>Gordon</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>(903) 894-6418</t>
+          <t>(903) 526-7419</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr"/>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Accurate Roof Systems</t>
+          <t>East Texas Roof Works &amp; Sheet Metal</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Barbara</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Jimenez</t>
+          <t>Gordon</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>(903) 894-6418</t>
+          <t>(903) 526-7419</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr"/>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Accurate Roof Systems</t>
+          <t>East Texas Roof Works &amp; Sheet Metal</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Director of Marketing</t>
+          <t>Corporate Secretary</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Zach</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Reilly</t>
+          <t>Rhodes</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2295,19 +2295,15 @@
           <t>(903) 258-1210</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>office.cxrroofing@gmail.com</t>
-        </is>
-      </c>
+      <c r="D53" s="2" t="inlineStr"/>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>CXR Roofing</t>
+          <t>Evolution Roofing LLC</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -2319,32 +2315,28 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Ricardo</t>
+          <t>Zachary</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Gamboa</t>
+          <t>Reilly</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>(903) 399-5403</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>contact@roof.care</t>
-        </is>
-      </c>
+          <t>(903) 258-1210</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr"/>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Roof Care Inc.</t>
+          <t>Evolution Roofing LLC</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -2356,32 +2348,32 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Michelle</t>
+          <t>Blake</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Gamboa</t>
+          <t>Wilabay</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>(903) 399-5403</t>
+          <t>(903) 320-3030</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>contact@roof.care</t>
+          <t>bxcroofing@yahoo.com</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Roof Care Inc.</t>
+          <t>BXC Roofing LLC</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Operations Director</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -2393,28 +2385,32 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Chris</t>
+          <t>Amelia</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Pratka</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>(903) 279-7000</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr"/>
+          <t>(903) 787-9043</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Info@roofmasterstyler.com</t>
+        </is>
+      </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Smith Roofing and Construction</t>
+          <t>Texas Roof Masters Tyler LLC</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Owner / Founder</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -2426,56 +2422,56 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Landon</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Stokes</t>
+          <t>Spencer</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>(682) 235-2880</t>
+          <t>(903) 894-6418</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr"/>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Hail King Professional Roofing LLC</t>
+          <t>Accurate Roof Systems</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Co-Owner / Founder</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Flint</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Lori</t>
+          <t>Melissa</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Anderson-Stokes</t>
+          <t>Spencer</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>(682) 235-2880</t>
+          <t>(903) 894-6418</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr"/>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Hail King Professional Roofing LLC</t>
+          <t>Accurate Roof Systems</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2485,60 +2481,72 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Flint</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Roman</t>
+          <t>David</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Skylar</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr"/>
+          <t>Jimenez</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>(903) 894-6418</t>
+        </is>
+      </c>
       <c r="D59" s="2" t="inlineStr"/>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Sky High Roofing</t>
+          <t>Accurate Roof Systems</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Director of Marketing</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Flint</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Hugo</t>
+          <t>Zach</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Escobar</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr"/>
-      <c r="D60" s="2" t="inlineStr"/>
+          <t>Reilly</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>(903) 258-1210</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>office.cxrroofing@gmail.com</t>
+        </is>
+      </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Sky High Roofing</t>
+          <t>CXR Roofing</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -2550,19 +2558,27 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Nick</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr"/>
+          <t>Ricardo</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Gamboa</t>
+        </is>
+      </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>(903) 714-3729</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr"/>
+          <t>(903) 399-5403</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>contact@roof.care</t>
+        </is>
+      </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Calvary Roofing and Construction</t>
+          <t>Roof Care Inc.</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -2572,63 +2588,67 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Lindale</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>April</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr"/>
+          <t>Michelle</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Gamboa</t>
+        </is>
+      </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>(903) 714-3729</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr"/>
+          <t>(903) 399-5403</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>contact@roof.care</t>
+        </is>
+      </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Calvary Roofing and Construction</t>
+          <t>Roof Care Inc.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Operations Director</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Lindale</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Ronnie</t>
+          <t>Chris</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Myers</t>
+          <t>Smith</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>(903) 573-3431</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>RonMyersRoofing@gmail.com</t>
-        </is>
-      </c>
+          <t>(903) 279-7000</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr"/>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Myers Roofing Solutions</t>
+          <t>Smith Roofing and Construction</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2638,67 +2658,63 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Lindale</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Steve</t>
+          <t>Landon</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Rohus</t>
+          <t>Stokes</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>(903) 839-2060</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>steverohus@gmail.com</t>
-        </is>
-      </c>
+          <t>(682) 235-2880</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr"/>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Steve's Quality Roofing</t>
+          <t>Hail King Professional Roofing LLC</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Whitehouse</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Cori</t>
+          <t>Lori</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Moore</t>
+          <t>Anderson-Stokes</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>(903) 534-3979</t>
+          <t>(682) 235-2880</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr"/>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Project One Roofing</t>
+          <t>Hail King Professional Roofing LLC</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2708,68 +2724,60 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Whitehouse</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>John Oliver</t>
+          <t>Roman</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Boyd II</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>(903) 810-7770</t>
-        </is>
-      </c>
+          <t>Skylar</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr"/>
       <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Boyd's of Texas</t>
+          <t>Sky High Roofing</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Bullard</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Kurt</t>
+          <t>Hugo</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Coleman</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>(903) 530-0350</t>
-        </is>
-      </c>
+          <t>Escobar</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="2" t="inlineStr"/>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Coleman Roofing</t>
+          <t>Sky High Roofing</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -2781,23 +2789,19 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Dayton</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Longfellow</t>
-        </is>
-      </c>
+          <t>Nick</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr"/>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>(903) 245-2988</t>
+          <t>(903) 714-3729</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Goodfella's Roofing</t>
+          <t>Calvary Roofing and Construction</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -2807,63 +2811,63 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Whitehouse</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Cody</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>Savell</t>
-        </is>
-      </c>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr"/>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>(903) 363-4140</t>
+          <t>(903) 714-3729</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr"/>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Bad Bear Roofing &amp; Construction</t>
+          <t>Calvary Roofing and Construction</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Roy</t>
+          <t>Ronnie</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Drewett</t>
+          <t>Myers</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>(903) 724-1511</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr"/>
+          <t>(903) 573-3431</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>RonMyersRoofing@gmail.com</t>
+        </is>
+      </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Premier Roofing ETX</t>
+          <t>Myers Roofing Solutions</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -2873,75 +2877,289 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr"/>
-      <c r="B71" s="2" t="inlineStr"/>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Steve</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Rohus</t>
+        </is>
+      </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>(903) 969-0503</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr"/>
+          <t>(903) 839-2060</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>steverohus@gmail.com</t>
+        </is>
+      </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>ETX Roofing &amp; Construction</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr"/>
+          <t>Steve's Quality Roofing</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Troup</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr"/>
-      <c r="B72" s="2" t="inlineStr"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Cori</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Moore</t>
+        </is>
+      </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>(903) 939-3168</t>
+          <t>(903) 534-3979</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr"/>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Advantage Roofing</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr"/>
+          <t>Project One Roofing</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Co-Owner</t>
+        </is>
+      </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr"/>
-      <c r="B73" s="2" t="inlineStr"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>John Oliver</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Boyd II</t>
+        </is>
+      </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>(903) 343-5700</t>
+          <t>(903) 810-7770</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
+          <t>Boyd's of Texas</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Bullard</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Kurt</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Coleman</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>(903) 530-0350</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Coleman Roofing</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Dayton</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Longfellow</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>(903) 245-2988</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr"/>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Goodfella's Roofing</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Whitehouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Cody</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Savell</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>(903) 363-4140</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr"/>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Bad Bear Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Flint</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Roy</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Drewett</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>(903) 724-1511</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr"/>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Premier Roofing ETX</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Tyler</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr"/>
+      <c r="B78" s="2" t="inlineStr"/>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>(903) 969-0503</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr"/>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>ETX Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Troup</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr"/>
+      <c r="B79" s="2" t="inlineStr"/>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>(903) 343-5700</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr"/>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
           <t>ValueGuard Roofing</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr"/>
-      <c r="G73" s="2" t="inlineStr">
+      <c r="F79" s="2" t="inlineStr"/>
+      <c r="G79" s="2" t="inlineStr">
         <is>
           <t>Flint</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G73"/>
+  <autoFilter ref="A1:G79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rebuild Smith County roofing contacts via /scrape-contacts skill (80 contacts, 45 companies, 9 cities)
New contacts found: Cable's Roofing, Project One Roofing (6 employees), Boyd's of Texas
(4 employees), Guardian Roofing Pros, Reliant Roofing, Firehouse Roofing, Roofing ETX,
Tyler Roof Repair, J W Roofing, Busby's Roofing, Noble Roofing, Bison Construction,
plus new emails for Tyler Roofing Co and Coleman Roofing.

https://claude.ai/code/session_019vJRSZ4rBkhi5FH5Wtx4Bj
</commit_message>
<xml_diff>
--- a/output/Smith_County_TX_Roofing_Contacts.xlsx
+++ b/output/Smith_County_TX_Roofing_Contacts.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Roofing Contacts Smith Co TX" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roofing Contacts Smith Co TX'!$A$1:$G$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roofing Contacts Smith Co TX'!$A$1:$G$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,16 +443,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -532,32 +532,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Shane</t>
+          <t>Darren</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Cable</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>(903) 765-7089</t>
+          <t>(903) 581-5599</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>cover3roofing@outlook.com</t>
+          <t>sales@cablesroofing.com</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Cover 3 Roofing and Construction</t>
+          <t>Cable's Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Owner / CEO</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -569,28 +569,32 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Eva</t>
+          <t>Macy</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Cable</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>(903) 765-7089</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
+          <t>(903) 581-5599</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>sales@cablesroofing.com</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Cover 3 Roofing and Construction</t>
+          <t>Cable's Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Co-Owner / Office Manager</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -602,32 +606,32 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>William</t>
+          <t>John</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Hill</t>
+          <t>Steele</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>(903) 630-4688</t>
+          <t>(903) 630-5751</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>contact@awhill.org</t>
+          <t>steeleroofingtyler@gmail.com</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>A&amp;W Hill Roofing &amp; Construction</t>
+          <t>Steele Roofing LLC</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -639,32 +643,28 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Ashley</t>
+          <t>Josiah</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Hill</t>
+          <t>Rosebury</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>(903) 630-4688</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>contact@awhill.org</t>
-        </is>
-      </c>
+          <t>(903) 326-7255</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>A&amp;W Hill Roofing &amp; Construction</t>
+          <t>Yosemite Roofing LLC</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Owner / Founder</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -676,27 +676,27 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>John Frank</t>
+          <t>Heath</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Adams III</t>
+          <t>Hicks</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>(903) 484-4231</t>
+          <t>(903) 534-8700</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>sales@adamsfamilyroofing.com</t>
+          <t>office@avcoroofing.com</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Adams Family Roofing</t>
+          <t>AVCO Roofing</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -706,76 +706,76 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Kassidy</t>
+          <t>Ronnie</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Adams</t>
+          <t>Lollar</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>(903) 484-4231</t>
+          <t>(903) 534-8700</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>sales@adamsfamilyroofing.com</t>
+          <t>office@avcoroofing.com</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Adams Family Roofing</t>
+          <t>AVCO Roofing</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Project Inspector</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Josiah</t>
+          <t>Bruce</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Rosebury</t>
+          <t>Webster</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>(903) 326-7255</t>
+          <t>(903) 534-8700</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>info@yosemiteroofing.com</t>
+          <t>office@avcoroofing.com</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Yosemite Roofing</t>
+          <t>AVCO Roofing</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Owner / Founder</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -787,69 +787,69 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Will</t>
+          <t>Emerald</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Miller</t>
+          <t>Bragg</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>(903) 920-6524</t>
+          <t>(903) 534-8700</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>tyler@priorityroofs.com</t>
+          <t>office@avcoroofing.com</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Priority Roofing</t>
+          <t>AVCO Roofing</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>CEO / Founder</t>
+          <t>Executive Assistant</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Lindale</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Faue</t>
+          <t>Admire</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>(903) 920-6524</t>
+          <t>(903) 780-7245</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>tyler@priorityroofs.com</t>
+          <t>jadmire@admireroofing.com</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Priority Roofing</t>
+          <t>Admire Roofing LLC</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Managing Partner</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -861,28 +861,32 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Micah</t>
+          <t>Shon</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>McQueen</t>
+          <t>Dickson</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>(903) 920-6524</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
+          <t>(903) 508-5011</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>sales@dicksonroofs.com</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Priority Roofing</t>
+          <t>Dickson Roofing</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Vice President</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -894,28 +898,32 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Cody</t>
+          <t>Talya</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Wilcox</t>
+          <t>Dickson</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>(903) 920-6524</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
+          <t>(903) 508-5011</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>sales@dicksonroofs.com</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Priority Roofing</t>
+          <t>Dickson Roofing</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Office Manager</t>
+          <t>Director of Marketing</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -927,61 +935,69 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Myrick</t>
+          <t>Cheri</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Prince</t>
+          <t>Dickson</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>(903) 437-7049</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
+          <t>(903) 508-5011</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>sales@dicksonroofs.com</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Redline Roofing &amp; Construction</t>
+          <t>Dickson Roofing</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Office Manager</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Lindale</t>
+          <t>Tyler</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Andrew Allan</t>
+          <t>Tommy Ray</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Quick</t>
+          <t>Sukiennik</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>(903) 505-5720</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
+          <t>(903) 597-4152</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>tylerroofingco@gmail.com</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Quick Roofing &amp; Restoration</t>
+          <t>Tyler Roofing Company Inc.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>President</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -993,28 +1009,32 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Billy</t>
+          <t>Mark</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Hargrove</t>
+          <t>Sukiennik</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>(903) 747-8206</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
+          <t>(903) 597-4152</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>MarkSukiennik@suddenlink.net</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Hargrove Roofing &amp; Construction</t>
+          <t>Tyler Roofing Company Inc.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1026,28 +1046,32 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Clyde</t>
+          <t>Cris</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Hargrove</t>
+          <t>Sukiennik</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>(903) 412-2710</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
+          <t>(903) 597-4152</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>tylerroofingco@gmail.com</t>
+        </is>
+      </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Hargrove Roofing &amp; Construction</t>
+          <t>Tyler Roofing Company Inc.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>General Manager</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1059,28 +1083,32 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Mae</t>
+          <t>Tracy</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Hargrove</t>
+          <t>Sukiennik</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>(903) 412-2710</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
+          <t>(903) 597-4152</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>tylerroofingco@gmail.com</t>
+        </is>
+      </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Hargrove Roofing &amp; Construction</t>
+          <t>Tyler Roofing Company Inc.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>Office Manager</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1092,28 +1120,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Jordan Zachary</t>
+          <t>Shane</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Cagle</t>
+          <t>Day</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>(903) 412-2710</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
+          <t>(903) 765-7089</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>cover3roofing@gmail.com</t>
+        </is>
+      </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Hargrove Roofing &amp; Construction</t>
+          <t>Cover 3 Roofing and Construction</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Branch Director</t>
+          <t>Co-Owner / CEO</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1125,28 +1157,32 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Devin</t>
+          <t>Eva</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Angel</t>
+          <t>Day</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>(903) 412-2710</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
+          <t>(903) 765-7089</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>cover3roofing@gmail.com</t>
+        </is>
+      </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Hargrove Roofing &amp; Construction</t>
+          <t>Cover 3 Roofing and Construction</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Tyler Sales Manager</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1158,32 +1194,32 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Shon</t>
+          <t>Kyle</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Dickson</t>
+          <t>Needham</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>(903) 508-5011</t>
+          <t>(903) 363-9155</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>sales@dicksonroofs.com</t>
+          <t>info@indemnityroofing.net</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Dickson Roofing</t>
+          <t>Indemnity Roofing Inc.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Co-Owner / Founder</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1195,32 +1231,32 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Talya</t>
+          <t>Josh</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Dickson</t>
+          <t>Hays</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>(903) 508-5011</t>
+          <t>(903) 363-9155</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>sales@dicksonroofs.com</t>
+          <t>info@indemnityroofing.net</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Dickson Roofing</t>
+          <t>Indemnity Roofing Inc.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Director of Marketing</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1232,32 +1268,28 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Cheri</t>
+          <t>Blake</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Dickson</t>
+          <t>Wilabay</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>(903) 508-5011</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>sales@dicksonroofs.com</t>
-        </is>
-      </c>
+          <t>(903) 320-3030</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Dickson Roofing</t>
+          <t>BXC Roofing LLC</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Office Manager</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1269,32 +1301,28 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Jonathan</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Admire</t>
+          <t>Weaver</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>(903) 780-7245</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>jadmire@admireroofing.com</t>
-        </is>
-      </c>
+          <t>(903) 592-5892</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Admire Roofing LLC</t>
+          <t>Weaver Action Roofing Company</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Owner / President</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1306,32 +1334,28 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Kyle</t>
+          <t>Janet</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Needham</t>
+          <t>Weaver</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>(903) 363-9155</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>info@indemnityroofing.net</t>
-        </is>
-      </c>
+          <t>(903) 592-5892</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Indemnity Roofing Inc.</t>
+          <t>Weaver Action Roofing Company</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner / Founder</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1343,27 +1367,27 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Josh</t>
+          <t>Ashley</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Hays</t>
+          <t>Hill</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>(903) 363-9155</t>
+          <t>(903) 630-4688</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>info@indemnityroofing.net</t>
+          <t>contact@awhill.org</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Indemnity Roofing Inc.</t>
+          <t>A&amp;W Hill Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1380,32 +1404,32 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Heath</t>
+          <t>William</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Hicks</t>
+          <t>Hill</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>(903) 534-8700</t>
+          <t>(903) 630-4688</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>office@avcoroofing.com</t>
+          <t>contact@awhill.org</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>AVCO Roofing</t>
+          <t>A&amp;W Hill Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1417,32 +1441,28 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Ronnie</t>
+          <t>Andrew</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Lollar</t>
+          <t>Quick</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>(903) 534-8700</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>office@avcoroofing.com</t>
-        </is>
-      </c>
+          <t>(903) 505-5720</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>AVCO Roofing</t>
+          <t>Quick Roofing &amp; Restoration LLC</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -1454,32 +1474,28 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Bruce</t>
+          <t>Landon</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Webster</t>
+          <t>Stokes</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>(903) 534-8700</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>office@avcoroofing.com</t>
-        </is>
-      </c>
+          <t>(682) 235-2880</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>AVCO Roofing</t>
+          <t>Hail King Professional Roofing LLC</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1491,32 +1507,28 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Emerald</t>
+          <t>Lori</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Bragg</t>
+          <t>Anderson-Stokes</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>(903) 534-8700</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>office@avcoroofing.com</t>
-        </is>
-      </c>
+          <t>(682) 235-2880</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>AVCO Roofing</t>
+          <t>Hail King Professional Roofing LLC</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Executive Assistant</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1565,12 +1577,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Klint</t>
+          <t>Tina</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Koppel</t>
+          <t>Anders</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1590,7 +1602,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Office Manager</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -1602,32 +1614,28 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Tina</t>
+          <t>Billy</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Anders</t>
+          <t>Hargrove</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>(903) 363-9160</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>email@asaproofing.com</t>
-        </is>
-      </c>
+          <t>(903) 412-2710</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>ASAP Roofing</t>
+          <t>Hargrove Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Office Manager</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -1639,32 +1647,28 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Jordan Zachary</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Steele</t>
+          <t>Cagle</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>(903) 630-5751</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>steeleroofingtyler@gmail.com</t>
-        </is>
-      </c>
+          <t>(903) 412-2710</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Steele Roofing LLC</t>
+          <t>Hargrove Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Branch Director</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -1676,32 +1680,28 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Ramon</t>
+          <t>Devin</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Balderrama</t>
+          <t>Angel</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>(903) 570-5441</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>rbroofing@att.net</t>
-        </is>
-      </c>
+          <t>(903) 412-2710</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>R.B. Roofing LLC</t>
+          <t>Hargrove Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Sales Manager</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -1713,28 +1713,28 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Tommy</t>
+          <t>Matthew Hunter</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Sukiennik</t>
+          <t>Andrews</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>(903) 597-4152</t>
+          <t>(903) 710-4022</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Tyler Roofing Company Inc.</t>
+          <t>Texas Direct Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>President</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -1746,28 +1746,28 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Mark</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Sukiennik</t>
+          <t>Stephens</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>(903) 597-4152</t>
+          <t>(903) 710-4022</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Tyler Roofing Company Inc.</t>
+          <t>Texas Direct Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Vice President</t>
+          <t>Director of Marketing</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -1779,28 +1779,28 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Cris</t>
+          <t>Dewayne</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Sukiennik</t>
+          <t>Gordon</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>(903) 597-4152</t>
+          <t>(903) 526-7419</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Tyler Roofing Company Inc.</t>
+          <t>East Texas Roof Works &amp; Sheet Metal</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>General Manager</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -1812,28 +1812,28 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Tracy</t>
+          <t>Barbara</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Sukiennik</t>
+          <t>Gordon</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>(903) 597-4152</t>
+          <t>(903) 526-7419</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Tyler Roofing Company Inc.</t>
+          <t>East Texas Roof Works &amp; Sheet Metal</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Office Manager</t>
+          <t>Corporate Secretary</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -1845,28 +1845,28 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Weaver</t>
+          <t>Spencer</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>(903) 592-5892</t>
+          <t>(903) 894-6418</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Weaver Action Roofing Company</t>
+          <t>Accurate Roof Systems</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Owner / President</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -1878,23 +1878,23 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Janet</t>
+          <t>Melissa</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Weaver</t>
+          <t>Spencer</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>(903) 592-5892</t>
+          <t>(903) 894-6418</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Weaver Action Roofing Company</t>
+          <t>Accurate Roof Systems</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1911,28 +1911,28 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>A.J.</t>
+          <t>David</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Cook III</t>
+          <t>Jimenez</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>(903) 595-4567</t>
+          <t>(903) 894-6418</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Cook and Son Roofing LLC</t>
+          <t>Accurate Roof Systems</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Director of Marketing</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -1944,28 +1944,32 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Moriah</t>
+          <t>Chris</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>McClinton</t>
+          <t>Smith</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>(903) 595-4567</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr"/>
+          <t>(903) 279-7000</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Csmithsrc@gmail.com</t>
+        </is>
+      </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Cook and Son Roofing LLC</t>
+          <t>Smith Roofing and Construction</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Secretary</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -1977,32 +1981,32 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Stephanie</t>
+          <t>Justin Dale</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Osborn</t>
+          <t>Deason</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>(903) 534-8700</t>
+          <t>(903) 426-1151</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>office@avcoroofing.com</t>
+          <t>sales@RoofRepairTyler.com</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>AVCO Roofing</t>
+          <t>Tyler Roof Repair</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Chief Operations Officer</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2014,23 +2018,19 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Ryan</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Merrell</t>
-        </is>
-      </c>
+          <t>Justin</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>(903) 939-3168</t>
+          <t>(903) 520-4111</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr"/>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Advantage Roofing Company</t>
+          <t>Bison Construction Pros</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2047,23 +2047,23 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Matthew Hunter</t>
+          <t>Myrick Brett</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Andrews</t>
+          <t>Prince</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>(903) 710-4022</t>
+          <t>(903) 437-7049</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Texas Direct Roofing &amp; Construction</t>
+          <t>Redline Roofing Company</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2073,67 +2073,67 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Ryan</t>
+          <t>Scott</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Stephens</t>
+          <t>Prince</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>(903) 710-4022</t>
+          <t>(903) 437-7049</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Texas Direct Roofing &amp; Construction</t>
+          <t>Redline Roofing Company</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Director of Marketing</t>
+          <t>Owner (Operations)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Greg</t>
+          <t>Will</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Tryon</t>
+          <t>Miller</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>(903) 752-7177</t>
+          <t>(903) 920-6524</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>gtryon@roofmaxx.com</t>
+          <t>tyler@priorityroofs.com</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Roof Maxx of Tyler</t>
+          <t>Priority Roofing of East Texas</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2143,195 +2143,203 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Dewayne</t>
+          <t>John</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Gordon</t>
+          <t>Faue</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>(903) 526-7419</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr"/>
+          <t>(903) 920-6524</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>tyler@priorityroofs.com</t>
+        </is>
+      </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>East Texas Roof Works &amp; Sheet Metal</t>
+          <t>Priority Roofing of East Texas</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Owner / Founder</t>
+          <t>General Manager</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Steve</t>
+          <t>Micah</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>DeRaad</t>
+          <t>McQueen</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>(903) 526-7419</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr"/>
+          <t>(903) 920-6524</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>tyler@priorityroofs.com</t>
+        </is>
+      </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>East Texas Roof Works &amp; Sheet Metal</t>
+          <t>Priority Roofing of East Texas</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Jimmy</t>
+          <t>Jay</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Gordon</t>
+          <t>Welling</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>(903) 526-7419</t>
+          <t>(903) 939-3168</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr"/>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>East Texas Roof Works &amp; Sheet Metal</t>
+          <t>Advantage Roofing Company</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>President</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Barbara</t>
+          <t>Mark</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Gordon</t>
+          <t>Latham</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>(903) 526-7419</t>
+          <t>(903) 817-0219</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr"/>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>East Texas Roof Works &amp; Sheet Metal</t>
+          <t>Firehouse Roofing</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Corporate Secretary</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Nicholas</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Rhodes</t>
+          <t>Gullatt</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>(903) 258-1210</t>
+          <t>(903) 714-3729</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr"/>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Evolution Roofing LLC</t>
+          <t>Calvary Roofing and Construction</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Zachary</t>
+          <t>April</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Reilly</t>
+          <t>Gullatt</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>(903) 258-1210</t>
+          <t>(903) 714-3729</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr"/>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Evolution Roofing LLC</t>
+          <t>Calvary Roofing and Construction</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2341,104 +2349,104 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Blake</t>
+          <t>Ronnie</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Wilabay</t>
+          <t>Myers</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>(903) 320-3030</t>
+          <t>(903) 573-3431</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>bxcroofing@yahoo.com</t>
+          <t>RonMyersRoofing@gmail.com</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>BXC Roofing LLC</t>
+          <t>Myers Roofing Solutions</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Lindale</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Amelia</t>
+          <t>Steve</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Pratka</t>
+          <t>Rohus</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>(903) 787-9043</t>
+          <t>(903) 839-2060</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Info@roofmasterstyler.com</t>
+          <t>steverohus@gmail.com</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Texas Roof Masters Tyler LLC</t>
+          <t>Steve's Quality Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Owner / Founder</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Gabriel</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Spencer</t>
+          <t>Moore</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>(903) 894-6418</t>
+          <t>(903) 534-3979</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr"/>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Accurate Roof Systems</t>
+          <t>Project One Roofing</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2448,30 +2456,30 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Melissa</t>
+          <t>Cori</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Spencer</t>
+          <t>Moore</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>(903) 894-6418</t>
+          <t>(903) 534-3979</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr"/>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Accurate Roof Systems</t>
+          <t>Project One Roofing</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2481,174 +2489,162 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Ted</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Jimenez</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>(903) 894-6418</t>
+          <t>(903) 534-3979</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr"/>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Accurate Roof Systems</t>
+          <t>Project One Roofing</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Director of Marketing</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Zach</t>
+          <t>Chris</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Reilly</t>
+          <t>Hughes</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>(903) 258-1210</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>office.cxrroofing@gmail.com</t>
-        </is>
-      </c>
+          <t>(903) 534-3979</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr"/>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>CXR Roofing</t>
+          <t>Project One Roofing</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Ricardo</t>
+          <t>Julia</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Gamboa</t>
+          <t>Hughes</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>(903) 399-5403</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>contact@roof.care</t>
-        </is>
-      </c>
+          <t>(903) 534-3979</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr"/>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Roof Care Inc.</t>
+          <t>Project One Roofing</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Insurance Agent</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Michelle</t>
+          <t>Meredith</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Gamboa</t>
+          <t>Bryans</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>(903) 399-5403</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>contact@roof.care</t>
-        </is>
-      </c>
+          <t>(903) 534-3979</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr"/>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Roof Care Inc.</t>
+          <t>Project One Roofing</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Operations Director</t>
+          <t>Marketing Director</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Chris</t>
+          <t>Dayton</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Longfellow</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>(903) 279-7000</t>
+          <t>(903) 245-2988</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr"/>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Smith Roofing and Construction</t>
+          <t>Goodfella's Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2658,216 +2654,232 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Landon</t>
+          <t>Macie</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Stokes</t>
+          <t>Longfellow</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>(682) 235-2880</t>
+          <t>(903) 245-2988</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr"/>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Hail King Professional Roofing LLC</t>
+          <t>Goodfella's Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Administrative Director</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Lori</t>
+          <t>Kurt</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Anderson-Stokes</t>
+          <t>Coleman</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>(682) 235-2880</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr"/>
+          <t>(903) 530-0350</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>kurt@colemanroofs.com</t>
+        </is>
+      </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Hail King Professional Roofing LLC</t>
+          <t>Coleman Roofing LLC</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Whitehouse</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Roman</t>
+          <t>John</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Skylar</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr"/>
+          <t>Boyd</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>(903) 810-7770</t>
+        </is>
+      </c>
       <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Sky High Roofing</t>
+          <t>Boyd's of Texas Contracting</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Owner / Director of Operations</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Bullard</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Hugo</t>
+          <t>Summer</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Escobar</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr"/>
+          <t>Boyd</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>(903) 810-7770</t>
+        </is>
+      </c>
       <c r="D67" s="2" t="inlineStr"/>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Sky High Roofing</t>
+          <t>Boyd's of Texas Contracting</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>Co-Founder / Director of Marketing</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Bullard</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Nick</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr"/>
+          <t>Christina</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Courville</t>
+        </is>
+      </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>(903) 714-3729</t>
+          <t>(903) 810-7770</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Calvary Roofing and Construction</t>
+          <t>Boyd's of Texas Contracting</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Office Manager</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Lindale</t>
+          <t>Bullard</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>April</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr"/>
+          <t>Danielle</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Sovia</t>
+        </is>
+      </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>(903) 714-3729</t>
+          <t>(903) 810-7770</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr"/>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Calvary Roofing and Construction</t>
+          <t>Boyd's of Texas Contracting</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Office Assistant</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Lindale</t>
+          <t>Bullard</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Ronnie</t>
+          <t>Jason</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Myers</t>
+          <t>Hadley</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>(903) 573-3431</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>RonMyersRoofing@gmail.com</t>
-        </is>
-      </c>
+          <t>(903) 707-3608</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr"/>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Myers Roofing Solutions</t>
+          <t>Reliant Roofing</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -2877,34 +2889,34 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Lindale</t>
+          <t>Bullard</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Steve</t>
+          <t>John Frank</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Rohus</t>
+          <t>Adams III</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>(903) 839-2060</t>
+          <t>(903) 484-4231</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>steverohus@gmail.com</t>
+          <t>sales@adamsfamilyroofing.com</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Steve's Quality Roofing</t>
+          <t>Adams Family Roofing LLC</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -2914,129 +2926,129 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Whitehouse</t>
+          <t>Flint</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Cori</t>
+          <t>Cody</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Moore</t>
+          <t>Savell</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>(903) 534-3979</t>
+          <t>(903) 363-4140</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr"/>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Project One Roofing</t>
+          <t>Bad Bear Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Co-Owner</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Whitehouse</t>
+          <t>Flint</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>John Oliver</t>
+          <t>Valeri</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Boyd II</t>
+          <t>Savell</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>(903) 810-7770</t>
+          <t>(903) 363-4140</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Boyd's of Texas</t>
+          <t>Bad Bear Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Co-Founder</t>
+          <t>Co-Owner</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Bullard</t>
+          <t>Flint</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Kurt</t>
+          <t>Richard Shelby</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Coleman</t>
+          <t>Henley</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>(903) 530-0350</t>
+          <t>(903) 710-3132</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr"/>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Coleman Roofing</t>
+          <t>Guardian Roofing Pros</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>President / Owner</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Flint</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Dayton</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>Longfellow</t>
-        </is>
-      </c>
+          <t>Jonathan</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr"/>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>(903) 245-2988</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr"/>
+          <t>(903) 312-7145</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>jonathan@roofingetx.com</t>
+        </is>
+      </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Goodfella's Roofing</t>
+          <t>Roofing ETX</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -3046,30 +3058,26 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Whitehouse</t>
+          <t>Flint</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Cody</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>Savell</t>
-        </is>
-      </c>
+          <t>Jonathan</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr"/>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>(903) 363-4140</t>
+          <t>(903) 343-5700</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr"/>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Bad Bear Roofing &amp; Construction</t>
+          <t>ValueGuard Roofing</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3086,23 +3094,19 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Roy</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>Drewett</t>
-        </is>
-      </c>
+          <t>Adrian</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr"/>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>(903) 724-1511</t>
+          <t>(903) 969-0503</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr"/>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Premier Roofing ETX</t>
+          <t>ETX Roofing &amp; Construction</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -3112,54 +3116,132 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Troup</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr"/>
-      <c r="B78" s="2" t="inlineStr"/>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Jerry</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Whitley</t>
+        </is>
+      </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>(903) 969-0503</t>
+          <t>(903) 371-1730</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr"/>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>ETX Roofing &amp; Construction</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr"/>
+          <t>J W Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Troup</t>
+          <t>Winona</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr"/>
-      <c r="B79" s="2" t="inlineStr"/>
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Dale</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Busby</t>
+        </is>
+      </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>(903) 343-5700</t>
+          <t>(903) 877-3100</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr"/>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>ValueGuard Roofing</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr"/>
+          <t>Busby's Roofing</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Flint</t>
+          <t>Winona</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Roy</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Drewett</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>(903) 724-1511</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr"/>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Premier Roofing of East Texas</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>New Chapel Hill</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr"/>
+      <c r="B81" s="2" t="inlineStr"/>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>(903) 738-4591</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr"/>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Noble Roofing</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Arp</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G79"/>
+  <autoFilter ref="A1:G81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>